<commit_message>
fix: validate wayback archive cli inputs
</commit_message>
<xml_diff>
--- a/research/wayback-archive-feature-audit.xlsx
+++ b/research/wayback-archive-feature-audit.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rc03453bb202842f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stories" sheetId="2" r:id="R95d101a016ea436e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Issues" sheetId="3" r:id="R22f1b9fbeae8419d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R8d37ce3e058f4e01"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stories" sheetId="2" r:id="R959189af79864a26"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Issues" sheetId="3" r:id="R8d5bdc7dc02345e3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -407,7 +407,7 @@
         <x:v>Current Loop</x:v>
       </x:c>
       <x:c r="B7" s="6" t="str">
-        <x:v>Story inventory created from code; manual and unit evidence logged; compare explicit-timestamp regression fixed and retested; further retest loop remains active.</x:v>
+        <x:v>Feature inventory is complete. All identified UX/logistical regressions have been fixed and retested; remaining open items are external Wayback dependency risks.</x:v>
       </x:c>
       <x:c r="C7" s="6"/>
       <x:c r="D7" s="6"/>
@@ -447,15 +447,15 @@
         <x:v>Pass</x:v>
       </x:c>
       <x:c r="B11" s="14" t="n">
-        <x:f>COUNTIF(Stories!I2:I29,"Pass")</x:f>
-        <x:v>18</x:v>
+        <x:f>COUNTIF(Stories!I2:I32,"Pass")</x:f>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="C11" s="6"/>
       <x:c r="D11" s="15" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="E11" s="15" t="n">
-        <x:f>COUNTIF(Issues!C2:C6,"Open")</x:f>
+        <x:f>COUNTIF(Issues!C2:C7,"Open")</x:f>
         <x:v>2</x:v>
       </x:c>
     </x:row>
@@ -464,7 +464,7 @@
         <x:v>Pass - External Risk</x:v>
       </x:c>
       <x:c r="B12" s="14" t="n">
-        <x:f>COUNTIF(Stories!I2:I29,"Pass - External Risk")</x:f>
+        <x:f>COUNTIF(Stories!I2:I32,"Pass - External Risk")</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="C12" s="6"/>
@@ -472,8 +472,8 @@
         <x:v>Resolved</x:v>
       </x:c>
       <x:c r="E12" s="15" t="n">
-        <x:f>COUNTIF(Issues!C2:C6,"Resolved")</x:f>
-        <x:v>3</x:v>
+        <x:f>COUNTIF(Issues!C2:C7,"Resolved")</x:f>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -481,16 +481,16 @@
         <x:v>Unit Only</x:v>
       </x:c>
       <x:c r="B13" s="14" t="n">
-        <x:f>COUNTIF(Stories!I2:I29,"Unit Only")</x:f>
-        <x:v>5</x:v>
+        <x:f>COUNTIF(Stories!I2:I32,"Unit Only")</x:f>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C13" s="6"/>
       <x:c r="D13" s="15" t="str">
         <x:v>Manual Stories Verified</x:v>
       </x:c>
       <x:c r="E13" s="15" t="n">
-        <x:f>COUNTIF(Stories!I2:I29,"Pass")+COUNTIF(Stories!I2:I29,"Pass - External Risk")</x:f>
-        <x:v>23</x:v>
+        <x:f>COUNTIF(Stories!I2:I32,"Pass")+COUNTIF(Stories!I2:I32,"Pass - External Risk")</x:f>
+        <x:v>27</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -498,7 +498,7 @@
         <x:v>Untested</x:v>
       </x:c>
       <x:c r="B14" s="14" t="n">
-        <x:f>COUNTIF(Stories!I2:I29,"Untested")</x:f>
+        <x:f>COUNTIF(Stories!I2:I32,"Untested")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C14" s="6"/>
@@ -506,7 +506,7 @@
         <x:v>Stories Needing More Work</x:v>
       </x:c>
       <x:c r="E14" s="15" t="n">
-        <x:f>COUNTIF(Stories!I2:I29,"Untested")+COUNTIF(Stories!I2:I29,"Fail")+COUNTIF(Stories!I2:I29,"Fixed Pending Retest")</x:f>
+        <x:f>COUNTIF(Stories!I2:I32,"Untested")+COUNTIF(Stories!I2:I32,"Fail")+COUNTIF(Stories!I2:I32,"Fixed Pending Retest")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -515,7 +515,7 @@
         <x:v>Fail</x:v>
       </x:c>
       <x:c r="B15" s="14" t="n">
-        <x:f>COUNTIF(Stories!I2:I29,"Fail")</x:f>
+        <x:f>COUNTIF(Stories!I2:I32,"Fail")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C15" s="6"/>
@@ -523,8 +523,8 @@
         <x:v>Stories Covered by Tests Only</x:v>
       </x:c>
       <x:c r="E15" s="15" t="n">
-        <x:f>COUNTIF(Stories!I2:I29,"Unit Only")</x:f>
-        <x:v>5</x:v>
+        <x:f>COUNTIF(Stories!I2:I32,"Unit Only")</x:f>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -532,7 +532,7 @@
         <x:v>Fixed Pending Retest</x:v>
       </x:c>
       <x:c r="B16" s="14" t="n">
-        <x:f>COUNTIF(Stories!I2:I29,"Fixed Pending Retest")</x:f>
+        <x:f>COUNTIF(Stories!I2:I32,"Fixed Pending Retest")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C16" s="6"/>
@@ -828,7 +828,7 @@
         <x:v>No direct unit test for CLI path</x:v>
       </x:c>
       <x:c r="H8" s="19" t="str">
-        <x:v>Manual batch run with `--input tmp/wayback_archive_audit/test_urls.txt` returned one saved result for example.com.</x:v>
+        <x:v>Manual batch run with `--input tests/fixtures/wayback_archive/urls_with_comments.txt` returned one processed result entry sourced from the file.</x:v>
       </x:c>
       <x:c r="I8" s="20" t="str">
         <x:v>Pass</x:v>
@@ -858,7 +858,7 @@
         <x:v>No direct unit test</x:v>
       </x:c>
       <x:c r="H9" s="19" t="str">
-        <x:v>Manual batch run with one positional example.com plus duplicate file entries returned `total: 1`.</x:v>
+        <x:v>Manual batch run with duplicate example.com entries in `tests/fixtures/wayback_archive/urls_with_comments.txt` returned `total: 1`.</x:v>
       </x:c>
       <x:c r="I9" s="20" t="str">
         <x:v>Pass</x:v>
@@ -948,10 +948,10 @@
         <x:v>test_read_url_file_skips_comments_and_blank_lines</x:v>
       </x:c>
       <x:c r="H12" s="19" t="str">
-        <x:v>Not manually executed through CLI yet.</x:v>
+        <x:v>Manual batch run against `tests/fixtures/wayback_archive/urls_with_comments.txt` processed only one URL, proving comments and blank lines were ignored.</x:v>
       </x:c>
       <x:c r="I12" s="20" t="str">
-        <x:v>Unit Only</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="J12" s="19" t="str"/>
     </x:row>
@@ -1316,7 +1316,7 @@
         <x:v>test_resolve_compare_pair_raises_when_both_timestamps_still_collapse</x:v>
       </x:c>
       <x:c r="H24" s="19" t="str">
-        <x:v>Not manually reproduced yet.</x:v>
+        <x:v>Covered by automated test that forces both timestamps to remain collapsed after CDX retry.</x:v>
       </x:c>
       <x:c r="I24" s="20" t="str">
         <x:v>Unit Only</x:v>
@@ -1346,7 +1346,7 @@
         <x:v>test_resolve_compare_pair_surfaces_cdx_disambiguation_failure</x:v>
       </x:c>
       <x:c r="H25" s="19" t="str">
-        <x:v>Not manually reproduced yet.</x:v>
+        <x:v>Covered by automated test that forces CDX disambiguation failure after collapsed availability results.</x:v>
       </x:c>
       <x:c r="I25" s="20" t="str">
         <x:v>Unit Only</x:v>
@@ -1406,7 +1406,7 @@
         <x:v>test_save_once_uses_http_error_location_header</x:v>
       </x:c>
       <x:c r="H27" s="19" t="str">
-        <x:v>No manual reproduction required.</x:v>
+        <x:v>Covered by automated test that simulates an HTTP error carrying a Wayback `Location` header.</x:v>
       </x:c>
       <x:c r="I27" s="20" t="str">
         <x:v>Unit Only</x:v>
@@ -1436,7 +1436,7 @@
         <x:v>test_save_once_uses_final_redirect_url</x:v>
       </x:c>
       <x:c r="H28" s="19" t="str">
-        <x:v>No manual reproduction required.</x:v>
+        <x:v>Covered by automated test that simulates a direct save redirect response.</x:v>
       </x:c>
       <x:c r="I28" s="20" t="str">
         <x:v>Unit Only</x:v>
@@ -1466,16 +1466,106 @@
         <x:v>Covered indirectly across all unit tests</x:v>
       </x:c>
       <x:c r="H29" s="19" t="str">
-        <x:v>Observed manually across save/available/batch-save/nearest/compare/history failure outputs.</x:v>
+        <x:v>Observed manually across save/available/batch-save/nearest/compare/history failure outputs, including newly validated input errors.</x:v>
       </x:c>
       <x:c r="I29" s="20" t="str">
         <x:v>Pass</x:v>
       </x:c>
       <x:c r="J29" s="19" t="str"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="19" t="str">
+        <x:v>US-029</x:v>
+      </x:c>
+      <x:c r="B30" s="19" t="str">
+        <x:v>available/history/nearest/compare</x:v>
+      </x:c>
+      <x:c r="C30" s="19" t="str">
+        <x:v>Reject malformed timestamp input</x:v>
+      </x:c>
+      <x:c r="D30" s="19" t="str">
+        <x:v>As a user, malformed timestamp values are rejected locally with a clear JSON error instead of causing a traceback or ambiguous network behavior.</x:v>
+      </x:c>
+      <x:c r="E30" s="19" t="str">
+        <x:v>Commands that accept timestamp flags return `{ error: ... }` when given a non-14-digit or impossible calendar timestamp.</x:v>
+      </x:c>
+      <x:c r="F30" s="19" t="str">
+        <x:v>validate_wayback_timestamp(); main() validation branches</x:v>
+      </x:c>
+      <x:c r="G30" s="19" t="str">
+        <x:v>test_validate_wayback_timestamp_rejects_non_14_digit_input; test_validate_wayback_timestamp_rejects_impossible_calendar_values</x:v>
+      </x:c>
+      <x:c r="H30" s="19" t="str">
+        <x:v>Manual `nearest https://example.com --timestamp nope`, `available https://example.com --timestamp nope`, and `history https://example.com --from-timestamp nope` each returned structured JSON errors.</x:v>
+      </x:c>
+      <x:c r="I30" s="20" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J30" s="19" t="str"/>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="19" t="str">
+        <x:v>US-030</x:v>
+      </x:c>
+      <x:c r="B31" s="19" t="str">
+        <x:v>compare</x:v>
+      </x:c>
+      <x:c r="C31" s="19" t="str">
+        <x:v>Reject partial explicit compare arguments</x:v>
+      </x:c>
+      <x:c r="D31" s="19" t="str">
+        <x:v>As a user, I cannot accidentally request explicit compare mode with only one timestamp argument.</x:v>
+      </x:c>
+      <x:c r="E31" s="19" t="str">
+        <x:v>Returns JSON error requiring both `--from-timestamp` and `--to-timestamp` together, or neither.</x:v>
+      </x:c>
+      <x:c r="F31" s="19" t="str">
+        <x:v>main() compare argument validation</x:v>
+      </x:c>
+      <x:c r="G31" s="19" t="str">
+        <x:v>test_main_compare_requires_both_explicit_timestamps</x:v>
+      </x:c>
+      <x:c r="H31" s="19" t="str">
+        <x:v>Manual `compare https://example.com --from-timestamp 20260101120000` returned the expected structured JSON error.</x:v>
+      </x:c>
+      <x:c r="I31" s="20" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J31" s="19" t="str"/>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="19" t="str">
+        <x:v>US-031</x:v>
+      </x:c>
+      <x:c r="B32" s="19" t="str">
+        <x:v>batch-save --input</x:v>
+      </x:c>
+      <x:c r="C32" s="19" t="str">
+        <x:v>Handle missing input file gracefully</x:v>
+      </x:c>
+      <x:c r="D32" s="19" t="str">
+        <x:v>As a user, a missing batch input file returns a structured JSON error instead of a Python traceback.</x:v>
+      </x:c>
+      <x:c r="E32" s="19" t="str">
+        <x:v>Returns `{ error: ... }` when the input file cannot be read.</x:v>
+      </x:c>
+      <x:c r="F32" s="19" t="str">
+        <x:v>read_url_file(); main() batch-save branch</x:v>
+      </x:c>
+      <x:c r="G32" s="19" t="str">
+        <x:v>test_read_url_file_raises_structured_error_for_missing_file</x:v>
+      </x:c>
+      <x:c r="H32" s="19" t="str">
+        <x:v>Manual `batch-save --input /Users/breno/Documents/code/PROJECTS/HRF_GRANT/freedom-skills/tmp/wayback_archive_comment_file.txt` returned a structured JSON error after the UX fix.</x:v>
+      </x:c>
+      <x:c r="I32" s="20" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="J32" s="19" t="str"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
-    <x:dataValidation type="list" sqref="I2:I29">
+    <x:dataValidation type="list" sqref="I2:I32">
       <x:formula1>"Pass,Pass - External Risk,Unit Only,Untested,Fail,Fixed Pending Retest"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -1634,6 +1724,29 @@
         <x:v>Fixed in current branch during this audit.</x:v>
       </x:c>
     </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="19" t="str">
+        <x:v>ISS-006</x:v>
+      </x:c>
+      <x:c r="B7" s="19" t="str">
+        <x:v>UX validation bug</x:v>
+      </x:c>
+      <x:c r="C7" s="19" t="str">
+        <x:v>Resolved</x:v>
+      </x:c>
+      <x:c r="D7" s="19" t="str">
+        <x:v>Malformed timestamps, missing batch input files, and partial explicit compare arguments previously produced tracebacks or silently triggered the wrong mode.</x:v>
+      </x:c>
+      <x:c r="E7" s="19" t="str">
+        <x:v>US-028, US-029, US-030, US-031</x:v>
+      </x:c>
+      <x:c r="F7" s="19" t="str">
+        <x:v>The wrapper now validates timestamp syntax, requires compare timestamps as a pair, and converts unreadable input files into structured JSON errors.</x:v>
+      </x:c>
+      <x:c r="G7" s="19" t="str">
+        <x:v>Reproduced manually, fixed in code, and retested through CLI and unit coverage.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>